<commit_message>
#33 Client and eSpark BOM added
</commit_message>
<xml_diff>
--- a/Design Files/Servo-Board-v1.0/BOM/eSpark-BOM-Servo-Board-v1.0.xlsx
+++ b/Design Files/Servo-Board-v1.0/BOM/eSpark-BOM-Servo-Board-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="646">
   <si>
     <t>Component list</t>
   </si>
@@ -1955,6 +1955,9 @@
   </si>
   <si>
     <t>C423076</t>
+  </si>
+  <si>
+    <t>C545497</t>
   </si>
 </sst>
 </file>
@@ -2309,7 +2312,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2447,6 +2450,12 @@
     <xf numFmtId="0" fontId="22" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2458,11 +2467,11 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2785,14 +2794,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="53"/>
-      <c r="L1" s="53"/>
-      <c r="M1" s="53"/>
-      <c r="N1" s="53"/>
-      <c r="O1" s="53"/>
-      <c r="P1" s="53"/>
-      <c r="Q1" s="53"/>
-      <c r="R1" s="53"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="55"/>
+      <c r="O1" s="55"/>
+      <c r="P1" s="55"/>
+      <c r="Q1" s="55"/>
+      <c r="R1" s="55"/>
     </row>
     <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -3090,7 +3099,7 @@
       <c r="H10" s="47" t="s">
         <v>409</v>
       </c>
-      <c r="I10" s="56" t="s">
+      <c r="I10" s="53" t="s">
         <v>621</v>
       </c>
       <c r="J10" s="47" t="s">
@@ -5094,7 +5103,7 @@
       <c r="N46" s="14">
         <v>50</v>
       </c>
-      <c r="O46" s="57" t="s">
+      <c r="O46" s="54" t="s">
         <v>623</v>
       </c>
       <c r="P46" s="15">
@@ -8077,8 +8086,8 @@
       </c>
       <c r="R100" s="14"/>
     </row>
-    <row r="101" spans="1:18" ht="36" x14ac:dyDescent="0.25">
-      <c r="A101" s="1"/>
+    <row r="101" spans="1:18" s="59" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A101" s="58"/>
       <c r="B101" s="17">
         <f t="shared" si="0"/>
         <v>94</v>
@@ -8156,7 +8165,9 @@
       <c r="H102" s="14" t="s">
         <v>409</v>
       </c>
-      <c r="I102" s="14"/>
+      <c r="I102" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J102" s="14" t="s">
         <v>541</v>
       </c>
@@ -8209,7 +8220,9 @@
       <c r="H103" s="20" t="s">
         <v>409</v>
       </c>
-      <c r="I103" s="20"/>
+      <c r="I103" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J103" s="20" t="s">
         <v>542</v>
       </c>
@@ -8262,7 +8275,9 @@
       <c r="H104" s="14" t="s">
         <v>446</v>
       </c>
-      <c r="I104" s="14"/>
+      <c r="I104" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J104" s="14" t="s">
         <v>543</v>
       </c>
@@ -8315,7 +8330,9 @@
       <c r="H105" s="20" t="s">
         <v>447</v>
       </c>
-      <c r="I105" s="20"/>
+      <c r="I105" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J105" s="20" t="s">
         <v>544</v>
       </c>
@@ -8368,8 +8385,12 @@
       <c r="H106" s="14" t="s">
         <v>448</v>
       </c>
-      <c r="I106" s="14"/>
-      <c r="J106" s="14"/>
+      <c r="I106" s="42" t="s">
+        <v>629</v>
+      </c>
+      <c r="J106" s="14" t="s">
+        <v>484</v>
+      </c>
       <c r="K106" s="44" t="s">
         <v>484</v>
       </c>
@@ -8380,14 +8401,18 @@
         <f>L106*5</f>
         <v>20</v>
       </c>
-      <c r="N106" s="14"/>
-      <c r="O106" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P106" s="15"/>
+      <c r="N106" s="14">
+        <v>21</v>
+      </c>
+      <c r="O106" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="P106" s="15">
+        <v>3.07789</v>
+      </c>
       <c r="Q106" s="15">
         <f>P106*N106</f>
-        <v>0</v>
+        <v>64.635689999999997</v>
       </c>
       <c r="R106" s="14"/>
     </row>
@@ -8415,7 +8440,9 @@
       <c r="H107" s="20" t="s">
         <v>449</v>
       </c>
-      <c r="I107" s="20"/>
+      <c r="I107" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J107" s="20" t="s">
         <v>545</v>
       </c>
@@ -8468,7 +8495,9 @@
       <c r="H108" s="14" t="s">
         <v>450</v>
       </c>
-      <c r="I108" s="14"/>
+      <c r="I108" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J108" s="14" t="s">
         <v>546</v>
       </c>
@@ -8521,7 +8550,9 @@
       <c r="H109" s="20" t="s">
         <v>449</v>
       </c>
-      <c r="I109" s="20"/>
+      <c r="I109" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J109" s="20" t="s">
         <v>547</v>
       </c>
@@ -8574,7 +8605,9 @@
       <c r="H110" s="14" t="s">
         <v>451</v>
       </c>
-      <c r="I110" s="14"/>
+      <c r="I110" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J110" s="14" t="s">
         <v>548</v>
       </c>
@@ -8627,7 +8660,9 @@
       <c r="H111" s="20" t="s">
         <v>449</v>
       </c>
-      <c r="I111" s="20"/>
+      <c r="I111" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J111" s="20" t="s">
         <v>549</v>
       </c>
@@ -8641,14 +8676,18 @@
         <f t="shared" ref="M111" si="98">L111*5</f>
         <v>25</v>
       </c>
-      <c r="N111" s="20"/>
-      <c r="O111" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P111" s="21"/>
+      <c r="N111" s="20">
+        <v>26</v>
+      </c>
+      <c r="O111" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="P111" s="21">
+        <v>3.4409999999999998</v>
+      </c>
       <c r="Q111" s="21">
         <f t="shared" ref="Q111" si="99">P111*N111</f>
-        <v>0</v>
+        <v>89.465999999999994</v>
       </c>
       <c r="R111" s="20"/>
     </row>
@@ -8676,7 +8715,9 @@
       <c r="H112" s="14" t="s">
         <v>449</v>
       </c>
-      <c r="I112" s="14"/>
+      <c r="I112" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J112" s="14" t="s">
         <v>550</v>
       </c>
@@ -8690,14 +8731,18 @@
         <f>L112*5</f>
         <v>20</v>
       </c>
-      <c r="N112" s="14"/>
-      <c r="O112" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P112" s="15"/>
+      <c r="N112" s="14">
+        <v>21</v>
+      </c>
+      <c r="O112" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="P112" s="15">
+        <v>0.31219999999999998</v>
+      </c>
       <c r="Q112" s="15">
         <f>P112*N112</f>
-        <v>0</v>
+        <v>6.5561999999999996</v>
       </c>
       <c r="R112" s="14"/>
     </row>
@@ -8725,7 +8770,9 @@
       <c r="H113" s="20" t="s">
         <v>447</v>
       </c>
-      <c r="I113" s="20"/>
+      <c r="I113" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J113" s="20" t="s">
         <v>551</v>
       </c>
@@ -8739,14 +8786,18 @@
         <f t="shared" ref="M113" si="100">L113*5</f>
         <v>20</v>
       </c>
-      <c r="N113" s="20"/>
-      <c r="O113" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P113" s="21"/>
+      <c r="N113" s="20">
+        <v>21</v>
+      </c>
+      <c r="O113" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="P113" s="21">
+        <v>1.4966999999999999</v>
+      </c>
       <c r="Q113" s="21">
         <f t="shared" ref="Q113" si="101">P113*N113</f>
-        <v>0</v>
+        <v>31.430699999999998</v>
       </c>
       <c r="R113" s="20"/>
     </row>
@@ -8774,8 +8825,12 @@
       <c r="H114" s="14" t="s">
         <v>449</v>
       </c>
-      <c r="I114" s="14"/>
-      <c r="J114" s="14"/>
+      <c r="I114" s="42" t="s">
+        <v>629</v>
+      </c>
+      <c r="J114" s="14" t="s">
+        <v>645</v>
+      </c>
       <c r="K114" s="44" t="s">
         <v>484</v>
       </c>
@@ -8786,14 +8841,18 @@
         <f>L114*5</f>
         <v>20</v>
       </c>
-      <c r="N114" s="14"/>
-      <c r="O114" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P114" s="15"/>
+      <c r="N114" s="14">
+        <v>21</v>
+      </c>
+      <c r="O114" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="P114" s="15">
+        <v>1.944</v>
+      </c>
       <c r="Q114" s="15">
         <f>P114*N114</f>
-        <v>0</v>
+        <v>40.823999999999998</v>
       </c>
       <c r="R114" s="14"/>
     </row>
@@ -8821,7 +8880,9 @@
       <c r="H115" s="20" t="s">
         <v>452</v>
       </c>
-      <c r="I115" s="20"/>
+      <c r="I115" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J115" s="14" t="s">
         <v>639</v>
       </c>
@@ -8874,7 +8935,9 @@
       <c r="H116" s="14" t="s">
         <v>452</v>
       </c>
-      <c r="I116" s="14"/>
+      <c r="I116" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J116" s="14" t="s">
         <v>552</v>
       </c>
@@ -8888,14 +8951,18 @@
         <f>L116*5</f>
         <v>40</v>
       </c>
-      <c r="N116" s="14"/>
-      <c r="O116" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P116" s="15"/>
+      <c r="N116" s="14">
+        <v>41</v>
+      </c>
+      <c r="O116" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="P116" s="15">
+        <v>1.1592</v>
+      </c>
       <c r="Q116" s="15">
         <f>P116*N116</f>
-        <v>0</v>
+        <v>47.527200000000001</v>
       </c>
       <c r="R116" s="14"/>
     </row>
@@ -8923,7 +8990,9 @@
       <c r="H117" s="20" t="s">
         <v>453</v>
       </c>
-      <c r="I117" s="20"/>
+      <c r="I117" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J117" s="20" t="s">
         <v>553</v>
       </c>
@@ -8937,14 +9006,18 @@
         <f t="shared" ref="M117" si="104">L117*5</f>
         <v>40</v>
       </c>
-      <c r="N117" s="20"/>
-      <c r="O117" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P117" s="21"/>
+      <c r="N117" s="20">
+        <v>41</v>
+      </c>
+      <c r="O117" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="P117" s="21">
+        <v>0.3</v>
+      </c>
       <c r="Q117" s="21">
         <f t="shared" ref="Q117" si="105">P117*N117</f>
-        <v>0</v>
+        <v>12.299999999999999</v>
       </c>
       <c r="R117" s="20"/>
     </row>
@@ -8972,7 +9045,9 @@
       <c r="H118" s="14" t="s">
         <v>454</v>
       </c>
-      <c r="I118" s="14"/>
+      <c r="I118" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J118" s="14" t="s">
         <v>554</v>
       </c>
@@ -8986,14 +9061,18 @@
         <f>L118*5</f>
         <v>20</v>
       </c>
-      <c r="N118" s="14"/>
-      <c r="O118" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P118" s="15"/>
+      <c r="N118" s="14">
+        <v>25</v>
+      </c>
+      <c r="O118" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="P118" s="15">
+        <v>6.83E-2</v>
+      </c>
       <c r="Q118" s="15">
         <f>P118*N118</f>
-        <v>0</v>
+        <v>1.7075</v>
       </c>
       <c r="R118" s="14"/>
     </row>
@@ -9021,7 +9100,9 @@
       <c r="H119" s="20" t="s">
         <v>455</v>
       </c>
-      <c r="I119" s="20"/>
+      <c r="I119" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J119" s="20" t="s">
         <v>555</v>
       </c>
@@ -9035,14 +9116,18 @@
         <f t="shared" ref="M119" si="106">L119*5</f>
         <v>80</v>
       </c>
-      <c r="N119" s="20"/>
-      <c r="O119" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P119" s="21"/>
+      <c r="N119" s="20">
+        <v>85</v>
+      </c>
+      <c r="O119" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="P119" s="21">
+        <v>0.11260000000000001</v>
+      </c>
       <c r="Q119" s="21">
         <f t="shared" ref="Q119" si="107">P119*N119</f>
-        <v>0</v>
+        <v>9.5709999999999997</v>
       </c>
       <c r="R119" s="20"/>
     </row>
@@ -9070,7 +9155,9 @@
       <c r="H120" s="50" t="s">
         <v>456</v>
       </c>
-      <c r="I120" s="50"/>
+      <c r="I120" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J120" s="50" t="s">
         <v>556</v>
       </c>
@@ -9084,16 +9171,21 @@
         <f>L120*5</f>
         <v>25</v>
       </c>
-      <c r="N120" s="51"/>
-      <c r="O120" s="14" t="s">
-        <v>623</v>
-      </c>
-      <c r="P120" s="51"/>
-      <c r="Q120" s="51">
-        <f>P120*N120</f>
-        <v>0</v>
-      </c>
-      <c r="R120" s="52"/>
+      <c r="N120" s="51" t="s">
+        <v>484</v>
+      </c>
+      <c r="O120" s="47" t="s">
+        <v>623</v>
+      </c>
+      <c r="P120" s="51" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q120" s="51" t="s">
+        <v>484</v>
+      </c>
+      <c r="R120" s="52" t="s">
+        <v>624</v>
+      </c>
     </row>
     <row r="121" spans="1:18" ht="24" x14ac:dyDescent="0.25">
       <c r="A121" s="1"/>
@@ -9119,7 +9211,9 @@
       <c r="H121" s="20" t="s">
         <v>457</v>
       </c>
-      <c r="I121" s="20"/>
+      <c r="I121" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J121" s="20" t="s">
         <v>557</v>
       </c>
@@ -9172,7 +9266,9 @@
       <c r="H122" s="14" t="s">
         <v>458</v>
       </c>
-      <c r="I122" s="14"/>
+      <c r="I122" s="42" t="s">
+        <v>629</v>
+      </c>
       <c r="J122" s="14" t="s">
         <v>558</v>
       </c>
@@ -9215,14 +9311,14 @@
       <c r="K123" s="1"/>
       <c r="L123" s="1"/>
       <c r="M123" s="1"/>
-      <c r="N123" s="54" t="s">
+      <c r="N123" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="O123" s="55"/>
-      <c r="P123" s="55"/>
-      <c r="Q123" s="18" t="e">
-        <f>SUM(#REF!)</f>
-        <v>#REF!</v>
+      <c r="O123" s="57"/>
+      <c r="P123" s="57"/>
+      <c r="Q123" s="18">
+        <f>SUM(Q8:Q122)</f>
+        <v>641.17748999999992</v>
       </c>
       <c r="R123" s="1"/>
     </row>
@@ -9240,14 +9336,14 @@
       <c r="K124" s="1"/>
       <c r="L124" s="1"/>
       <c r="M124" s="1"/>
-      <c r="N124" s="54" t="s">
+      <c r="N124" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="O124" s="55"/>
-      <c r="P124" s="55"/>
-      <c r="Q124" s="19" t="e">
+      <c r="O124" s="57"/>
+      <c r="P124" s="57"/>
+      <c r="Q124" s="19">
         <f>Q123/5</f>
-        <v>#REF!</v>
+        <v>128.23549799999998</v>
       </c>
       <c r="R124" s="1"/>
     </row>
@@ -9356,8 +9452,17 @@
     <hyperlink ref="O101" r:id="rId93"/>
     <hyperlink ref="O102" r:id="rId94"/>
     <hyperlink ref="O103" r:id="rId95"/>
+    <hyperlink ref="O106" r:id="rId96"/>
+    <hyperlink ref="O111" r:id="rId97"/>
+    <hyperlink ref="O112" r:id="rId98"/>
+    <hyperlink ref="O113" r:id="rId99"/>
+    <hyperlink ref="O114" r:id="rId100"/>
+    <hyperlink ref="O116" r:id="rId101"/>
+    <hyperlink ref="O117" r:id="rId102"/>
+    <hyperlink ref="O118" r:id="rId103"/>
+    <hyperlink ref="O119" r:id="rId104"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId96"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId105"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#35 eSpark and Client BOM added
</commit_message>
<xml_diff>
--- a/Design Files/Servo-Board-v1.0/BOM/eSpark-BOM-Servo-Board-v1.0.xlsx
+++ b/Design Files/Servo-Board-v1.0/BOM/eSpark-BOM-Servo-Board-v1.0.xlsx
@@ -2456,6 +2456,12 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2466,12 +2472,6 @@
     <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2794,14 +2794,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
+      <c r="O1" s="57"/>
+      <c r="P1" s="57"/>
+      <c r="Q1" s="57"/>
+      <c r="R1" s="57"/>
     </row>
     <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -3061,7 +3061,7 @@
         <v>45</v>
       </c>
       <c r="N9" s="14">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="O9" s="48" t="s">
         <v>623</v>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="Q9" s="21">
         <f t="shared" ref="Q9" si="2">P9*N9</f>
-        <v>0.41599999999999998</v>
+        <v>1.248</v>
       </c>
       <c r="R9" s="20"/>
     </row>
@@ -3612,7 +3612,7 @@
         <v>50</v>
       </c>
       <c r="N19" s="20">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="O19" s="48" t="s">
         <v>623</v>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="Q19" s="21">
         <f t="shared" ref="Q19" si="12">P19*N19</f>
-        <v>0.42</v>
+        <v>0.84</v>
       </c>
       <c r="R19" s="20"/>
     </row>
@@ -7693,10 +7693,12 @@
       <c r="O93" s="48" t="s">
         <v>623</v>
       </c>
-      <c r="P93" s="21"/>
+      <c r="P93" s="21">
+        <v>1E-3</v>
+      </c>
       <c r="Q93" s="21">
         <f t="shared" ref="Q93" si="82">P93*N93</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="R93" s="20"/>
     </row>
@@ -8086,8 +8088,8 @@
       </c>
       <c r="R100" s="14"/>
     </row>
-    <row r="101" spans="1:18" s="59" customFormat="1" ht="36" x14ac:dyDescent="0.25">
-      <c r="A101" s="58"/>
+    <row r="101" spans="1:18" s="56" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A101" s="55"/>
       <c r="B101" s="17">
         <f t="shared" si="0"/>
         <v>94</v>
@@ -9228,7 +9230,7 @@
         <v>25</v>
       </c>
       <c r="N121" s="20">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="O121" s="48" t="s">
         <v>623</v>
@@ -9238,7 +9240,7 @@
       </c>
       <c r="Q121" s="21">
         <f t="shared" ref="Q121" si="109">P121*N121</f>
-        <v>3.008</v>
+        <v>9.0240000000000009</v>
       </c>
       <c r="R121" s="20"/>
     </row>
@@ -9311,14 +9313,14 @@
       <c r="K123" s="1"/>
       <c r="L123" s="1"/>
       <c r="M123" s="1"/>
-      <c r="N123" s="56" t="s">
+      <c r="N123" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="O123" s="57"/>
-      <c r="P123" s="57"/>
+      <c r="O123" s="59"/>
+      <c r="P123" s="59"/>
       <c r="Q123" s="18">
         <f>SUM(Q8:Q122)</f>
-        <v>641.17748999999992</v>
+        <v>648.54548999999975</v>
       </c>
       <c r="R123" s="1"/>
     </row>
@@ -9336,14 +9338,14 @@
       <c r="K124" s="1"/>
       <c r="L124" s="1"/>
       <c r="M124" s="1"/>
-      <c r="N124" s="56" t="s">
+      <c r="N124" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="O124" s="57"/>
-      <c r="P124" s="57"/>
+      <c r="O124" s="59"/>
+      <c r="P124" s="59"/>
       <c r="Q124" s="19">
         <f>Q123/5</f>
-        <v>128.23549799999998</v>
+        <v>129.70909799999995</v>
       </c>
       <c r="R124" s="1"/>
     </row>
@@ -9368,99 +9370,99 @@
     <hyperlink ref="O17" r:id="rId9"/>
     <hyperlink ref="O18" r:id="rId10"/>
     <hyperlink ref="O19" r:id="rId11"/>
-    <hyperlink ref="O28" r:id="rId12"/>
-    <hyperlink ref="O29" r:id="rId13"/>
-    <hyperlink ref="O30" r:id="rId14"/>
-    <hyperlink ref="O31" r:id="rId15"/>
-    <hyperlink ref="O34" r:id="rId16"/>
-    <hyperlink ref="O36" r:id="rId17"/>
-    <hyperlink ref="O35" r:id="rId18"/>
-    <hyperlink ref="O37" r:id="rId19"/>
-    <hyperlink ref="O38" r:id="rId20"/>
-    <hyperlink ref="O39" r:id="rId21"/>
-    <hyperlink ref="O41" r:id="rId22"/>
-    <hyperlink ref="O42" r:id="rId23"/>
-    <hyperlink ref="O43" r:id="rId24"/>
-    <hyperlink ref="O44" r:id="rId25"/>
-    <hyperlink ref="O45" r:id="rId26"/>
-    <hyperlink ref="O46" r:id="rId27"/>
-    <hyperlink ref="O47" r:id="rId28"/>
-    <hyperlink ref="O49" r:id="rId29"/>
-    <hyperlink ref="O50" r:id="rId30"/>
-    <hyperlink ref="O51" r:id="rId31"/>
-    <hyperlink ref="O54" r:id="rId32"/>
-    <hyperlink ref="O55" r:id="rId33"/>
-    <hyperlink ref="O56" r:id="rId34"/>
-    <hyperlink ref="O57" r:id="rId35"/>
-    <hyperlink ref="O59" r:id="rId36"/>
-    <hyperlink ref="O61" r:id="rId37"/>
-    <hyperlink ref="O65" r:id="rId38"/>
-    <hyperlink ref="O66" r:id="rId39"/>
-    <hyperlink ref="O68" r:id="rId40"/>
-    <hyperlink ref="O69" r:id="rId41"/>
-    <hyperlink ref="O70" r:id="rId42"/>
-    <hyperlink ref="O71" r:id="rId43"/>
-    <hyperlink ref="O72" r:id="rId44"/>
-    <hyperlink ref="O73" r:id="rId45"/>
-    <hyperlink ref="O74" r:id="rId46"/>
-    <hyperlink ref="O75" r:id="rId47"/>
-    <hyperlink ref="O77" r:id="rId48"/>
-    <hyperlink ref="O76" r:id="rId49"/>
-    <hyperlink ref="O78" r:id="rId50"/>
-    <hyperlink ref="O79" r:id="rId51"/>
-    <hyperlink ref="O80" r:id="rId52"/>
-    <hyperlink ref="O81" r:id="rId53"/>
-    <hyperlink ref="O82" r:id="rId54"/>
-    <hyperlink ref="O94" r:id="rId55"/>
-    <hyperlink ref="O105" r:id="rId56"/>
-    <hyperlink ref="O104" r:id="rId57"/>
-    <hyperlink ref="O107" r:id="rId58"/>
-    <hyperlink ref="O108" r:id="rId59"/>
-    <hyperlink ref="O109" r:id="rId60"/>
-    <hyperlink ref="O110" r:id="rId61"/>
-    <hyperlink ref="O115" r:id="rId62"/>
-    <hyperlink ref="O121" r:id="rId63"/>
-    <hyperlink ref="O122" r:id="rId64"/>
-    <hyperlink ref="O20" r:id="rId65"/>
-    <hyperlink ref="O21" r:id="rId66"/>
-    <hyperlink ref="O22" r:id="rId67"/>
-    <hyperlink ref="O25" r:id="rId68"/>
-    <hyperlink ref="O26" r:id="rId69"/>
-    <hyperlink ref="O32" r:id="rId70"/>
-    <hyperlink ref="O33" r:id="rId71"/>
-    <hyperlink ref="O48" r:id="rId72"/>
-    <hyperlink ref="O52" r:id="rId73"/>
-    <hyperlink ref="O53" r:id="rId74"/>
-    <hyperlink ref="O60" r:id="rId75"/>
-    <hyperlink ref="O62" r:id="rId76"/>
-    <hyperlink ref="O63" r:id="rId77"/>
-    <hyperlink ref="O64" r:id="rId78"/>
-    <hyperlink ref="O83" r:id="rId79"/>
-    <hyperlink ref="O84" r:id="rId80"/>
-    <hyperlink ref="O85" r:id="rId81"/>
-    <hyperlink ref="O86" r:id="rId82"/>
-    <hyperlink ref="O87" r:id="rId83"/>
-    <hyperlink ref="O90" r:id="rId84"/>
-    <hyperlink ref="O91" r:id="rId85"/>
-    <hyperlink ref="O92" r:id="rId86"/>
-    <hyperlink ref="O93" r:id="rId87"/>
-    <hyperlink ref="O96" r:id="rId88"/>
-    <hyperlink ref="O97" r:id="rId89"/>
-    <hyperlink ref="O98" r:id="rId90"/>
-    <hyperlink ref="O99" r:id="rId91"/>
-    <hyperlink ref="O100" r:id="rId92"/>
-    <hyperlink ref="O101" r:id="rId93"/>
-    <hyperlink ref="O102" r:id="rId94"/>
-    <hyperlink ref="O103" r:id="rId95"/>
-    <hyperlink ref="O106" r:id="rId96"/>
-    <hyperlink ref="O111" r:id="rId97"/>
-    <hyperlink ref="O112" r:id="rId98"/>
-    <hyperlink ref="O113" r:id="rId99"/>
-    <hyperlink ref="O114" r:id="rId100"/>
-    <hyperlink ref="O116" r:id="rId101"/>
-    <hyperlink ref="O117" r:id="rId102"/>
-    <hyperlink ref="O118" r:id="rId103"/>
-    <hyperlink ref="O119" r:id="rId104"/>
+    <hyperlink ref="O29" r:id="rId12"/>
+    <hyperlink ref="O30" r:id="rId13"/>
+    <hyperlink ref="O31" r:id="rId14"/>
+    <hyperlink ref="O34" r:id="rId15"/>
+    <hyperlink ref="O36" r:id="rId16"/>
+    <hyperlink ref="O35" r:id="rId17"/>
+    <hyperlink ref="O37" r:id="rId18"/>
+    <hyperlink ref="O38" r:id="rId19"/>
+    <hyperlink ref="O39" r:id="rId20"/>
+    <hyperlink ref="O41" r:id="rId21"/>
+    <hyperlink ref="O42" r:id="rId22"/>
+    <hyperlink ref="O43" r:id="rId23"/>
+    <hyperlink ref="O44" r:id="rId24"/>
+    <hyperlink ref="O45" r:id="rId25"/>
+    <hyperlink ref="O46" r:id="rId26"/>
+    <hyperlink ref="O47" r:id="rId27"/>
+    <hyperlink ref="O49" r:id="rId28"/>
+    <hyperlink ref="O50" r:id="rId29"/>
+    <hyperlink ref="O51" r:id="rId30"/>
+    <hyperlink ref="O54" r:id="rId31"/>
+    <hyperlink ref="O55" r:id="rId32"/>
+    <hyperlink ref="O56" r:id="rId33"/>
+    <hyperlink ref="O57" r:id="rId34"/>
+    <hyperlink ref="O59" r:id="rId35"/>
+    <hyperlink ref="O61" r:id="rId36"/>
+    <hyperlink ref="O65" r:id="rId37"/>
+    <hyperlink ref="O66" r:id="rId38"/>
+    <hyperlink ref="O68" r:id="rId39"/>
+    <hyperlink ref="O69" r:id="rId40"/>
+    <hyperlink ref="O70" r:id="rId41"/>
+    <hyperlink ref="O71" r:id="rId42"/>
+    <hyperlink ref="O72" r:id="rId43"/>
+    <hyperlink ref="O73" r:id="rId44"/>
+    <hyperlink ref="O74" r:id="rId45"/>
+    <hyperlink ref="O75" r:id="rId46"/>
+    <hyperlink ref="O77" r:id="rId47"/>
+    <hyperlink ref="O76" r:id="rId48"/>
+    <hyperlink ref="O78" r:id="rId49"/>
+    <hyperlink ref="O79" r:id="rId50"/>
+    <hyperlink ref="O80" r:id="rId51"/>
+    <hyperlink ref="O81" r:id="rId52"/>
+    <hyperlink ref="O82" r:id="rId53"/>
+    <hyperlink ref="O94" r:id="rId54"/>
+    <hyperlink ref="O105" r:id="rId55"/>
+    <hyperlink ref="O104" r:id="rId56"/>
+    <hyperlink ref="O107" r:id="rId57"/>
+    <hyperlink ref="O108" r:id="rId58"/>
+    <hyperlink ref="O109" r:id="rId59"/>
+    <hyperlink ref="O110" r:id="rId60"/>
+    <hyperlink ref="O115" r:id="rId61"/>
+    <hyperlink ref="O121" r:id="rId62"/>
+    <hyperlink ref="O122" r:id="rId63"/>
+    <hyperlink ref="O20" r:id="rId64"/>
+    <hyperlink ref="O21" r:id="rId65"/>
+    <hyperlink ref="O22" r:id="rId66"/>
+    <hyperlink ref="O25" r:id="rId67"/>
+    <hyperlink ref="O26" r:id="rId68"/>
+    <hyperlink ref="O32" r:id="rId69"/>
+    <hyperlink ref="O33" r:id="rId70"/>
+    <hyperlink ref="O48" r:id="rId71"/>
+    <hyperlink ref="O52" r:id="rId72"/>
+    <hyperlink ref="O53" r:id="rId73"/>
+    <hyperlink ref="O60" r:id="rId74"/>
+    <hyperlink ref="O62" r:id="rId75"/>
+    <hyperlink ref="O63" r:id="rId76"/>
+    <hyperlink ref="O64" r:id="rId77"/>
+    <hyperlink ref="O83" r:id="rId78"/>
+    <hyperlink ref="O84" r:id="rId79"/>
+    <hyperlink ref="O85" r:id="rId80"/>
+    <hyperlink ref="O86" r:id="rId81"/>
+    <hyperlink ref="O87" r:id="rId82"/>
+    <hyperlink ref="O90" r:id="rId83"/>
+    <hyperlink ref="O91" r:id="rId84"/>
+    <hyperlink ref="O92" r:id="rId85"/>
+    <hyperlink ref="O93" r:id="rId86"/>
+    <hyperlink ref="O96" r:id="rId87"/>
+    <hyperlink ref="O97" r:id="rId88"/>
+    <hyperlink ref="O98" r:id="rId89"/>
+    <hyperlink ref="O99" r:id="rId90"/>
+    <hyperlink ref="O100" r:id="rId91"/>
+    <hyperlink ref="O101" r:id="rId92"/>
+    <hyperlink ref="O102" r:id="rId93"/>
+    <hyperlink ref="O103" r:id="rId94"/>
+    <hyperlink ref="O106" r:id="rId95"/>
+    <hyperlink ref="O111" r:id="rId96"/>
+    <hyperlink ref="O112" r:id="rId97"/>
+    <hyperlink ref="O113" r:id="rId98"/>
+    <hyperlink ref="O114" r:id="rId99"/>
+    <hyperlink ref="O116" r:id="rId100"/>
+    <hyperlink ref="O117" r:id="rId101"/>
+    <hyperlink ref="O118" r:id="rId102"/>
+    <hyperlink ref="O119" r:id="rId103"/>
+    <hyperlink ref="O28" r:id="rId104"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId105"/>

</xml_diff>